<commit_message>
Data: weekly refresh — sku_master, weekly sales, FBA shipments, inventory + Fossil
Refreshed inputs across the pipeline:
  - sku_master.xlsx (canonical)
  - weekly_sales_snapshot.csv
  - inventory_amazon_{nexlev, viomi, audio_array, WM}.csv
  - inventory_ledger_{nexlev, viomi, Audio Array, WM}.csv
  - fba_shipments_{nexlev, viomi, Audio Array, WM}.csv
  - Fossil Replenishment master + In-Transit/Open PO + FBA shipments + ledger

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/input/sku_master.xlsx
+++ b/data/input/sku_master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\master\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C6830BC-D0D3-4AA3-84B9-EE5C05804355}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A85C6266-F9AE-4AD6-AC76-677040D8152A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{117C6BDF-C413-4A9B-8C98-0B7CEC880D6C}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6332" uniqueCount="3041">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6333" uniqueCount="3042">
   <si>
     <t>FBA SKU</t>
   </si>
@@ -9160,6 +9160,9 @@
   </si>
   <si>
     <t>B0BVHZ5MKZ</t>
+  </si>
+  <si>
+    <t>B0H2FCK54H</t>
   </si>
 </sst>
 </file>
@@ -9270,7 +9273,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -9326,6 +9329,7 @@
     <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -37147,7 +37151,9 @@
         <v>2869</v>
       </c>
       <c r="B898" s="5"/>
-      <c r="C898" s="5"/>
+      <c r="C898" s="19" t="s">
+        <v>3041</v>
+      </c>
       <c r="D898" s="5" t="s">
         <v>521</v>
       </c>

</xml_diff>

<commit_message>
Data: refresh sku_master (917 rows) + CB Replenishment_Master
Pulled latest canonical sku_master from G:/.../FastAPI/data/master/.
Verified all 5 replenishment masters still align: 0 NotInMaster, 0
ModelMismatch, 0 ASINMismatch across CB/AA/WM/Nexlev/Viomi.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/input/sku_master.xlsx
+++ b/data/input/sku_master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\master\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A85C6266-F9AE-4AD6-AC76-677040D8152A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FE361CE-6714-46C3-BB2A-17E99E588D6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{117C6BDF-C413-4A9B-8C98-0B7CEC880D6C}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6333" uniqueCount="3042">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6336" uniqueCount="3045">
   <si>
     <t>FBA SKU</t>
   </si>
@@ -9163,6 +9163,15 @@
   </si>
   <si>
     <t>B0H2FCK54H</t>
+  </si>
+  <si>
+    <t>B0H2ZCQFTZ</t>
+  </si>
+  <si>
+    <t>B0H2Z6R6V8</t>
+  </si>
+  <si>
+    <t>B0H3LHF2WW</t>
   </si>
 </sst>
 </file>
@@ -9329,7 +9338,9 @@
     <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -36744,7 +36755,9 @@
         <v>2842</v>
       </c>
       <c r="B885" s="5"/>
-      <c r="C885" s="5"/>
+      <c r="C885" s="19" t="s">
+        <v>3042</v>
+      </c>
       <c r="D885" s="5" t="s">
         <v>521</v>
       </c>
@@ -36771,7 +36784,9 @@
         <v>2844</v>
       </c>
       <c r="B886" s="5"/>
-      <c r="C886" s="5"/>
+      <c r="C886" s="19" t="s">
+        <v>3043</v>
+      </c>
       <c r="D886" s="5" t="s">
         <v>521</v>
       </c>
@@ -37151,7 +37166,7 @@
         <v>2869</v>
       </c>
       <c r="B898" s="5"/>
-      <c r="C898" s="19" t="s">
+      <c r="C898" t="s">
         <v>3041</v>
       </c>
       <c r="D898" s="5" t="s">
@@ -37593,7 +37608,9 @@
         <v>3030</v>
       </c>
       <c r="B914" s="5"/>
-      <c r="C914" s="5"/>
+      <c r="C914" s="19" t="s">
+        <v>3044</v>
+      </c>
       <c r="D914" s="5" t="s">
         <v>521</v>
       </c>

</xml_diff>

<commit_message>
Fossil master + In-Transit PO refresh + sku_master update
- data/input/Fossil Replenishment/Fossil Replenishment.xlsx
- data/input/Fossil Replenishment/In-Transit_Open_PO_Fossil.xlsx
- data/input/sku_master.xlsx

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/input/sku_master.xlsx
+++ b/data/input/sku_master.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\AM - Inventory replenishment\AM_Replenishment\data\input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\master\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38349CF2-A5BD-4384-B53C-6283B92C9B73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A73E827F-C73A-42B0-B756-90949A21AEDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{117C6BDF-C413-4A9B-8C98-0B7CEC880D6C}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$M$3007</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$M$3009</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16784" uniqueCount="9300">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16934" uniqueCount="9390">
   <si>
     <t>FBA SKU</t>
   </si>
@@ -27937,6 +27937,276 @@
   </si>
   <si>
     <t>SP-02</t>
+  </si>
+  <si>
+    <t>FBA80220</t>
+  </si>
+  <si>
+    <t>B0GDKG6QRV</t>
+  </si>
+  <si>
+    <t>AR11742</t>
+  </si>
+  <si>
+    <t>FBA80221</t>
+  </si>
+  <si>
+    <t>B0GDX6M95H</t>
+  </si>
+  <si>
+    <t>AR11743</t>
+  </si>
+  <si>
+    <t>FBA80222</t>
+  </si>
+  <si>
+    <t>B0GHJMFM23</t>
+  </si>
+  <si>
+    <t>AR11763</t>
+  </si>
+  <si>
+    <t>FBA80223</t>
+  </si>
+  <si>
+    <t>B0GHD9GN9C</t>
+  </si>
+  <si>
+    <t>AR11769</t>
+  </si>
+  <si>
+    <t>FBA80224</t>
+  </si>
+  <si>
+    <t>B0GTC9238R</t>
+  </si>
+  <si>
+    <t>AX4300</t>
+  </si>
+  <si>
+    <t>FBA80225</t>
+  </si>
+  <si>
+    <t>B0GTC9PS5Z</t>
+  </si>
+  <si>
+    <t>AX7178SET</t>
+  </si>
+  <si>
+    <t>FBA80226</t>
+  </si>
+  <si>
+    <t>B07SV6HR8T</t>
+  </si>
+  <si>
+    <t>DZ2237</t>
+  </si>
+  <si>
+    <t>FBA80227</t>
+  </si>
+  <si>
+    <t>B07SW9C6ZH</t>
+  </si>
+  <si>
+    <t>DZ2239</t>
+  </si>
+  <si>
+    <t>FBA80228</t>
+  </si>
+  <si>
+    <t>B07SYFYGR6</t>
+  </si>
+  <si>
+    <t>DZ4711</t>
+  </si>
+  <si>
+    <t>FBA80229</t>
+  </si>
+  <si>
+    <t>B07SYSQJDN</t>
+  </si>
+  <si>
+    <t>DZ4712</t>
+  </si>
+  <si>
+    <t>FBA80230</t>
+  </si>
+  <si>
+    <t>B0GTC2MW2C</t>
+  </si>
+  <si>
+    <t>ES5473</t>
+  </si>
+  <si>
+    <t>FBA80231</t>
+  </si>
+  <si>
+    <t>B0GTC3BMTN</t>
+  </si>
+  <si>
+    <t>ES5477</t>
+  </si>
+  <si>
+    <t>FBA80232</t>
+  </si>
+  <si>
+    <t>B0GTC7QS9P</t>
+  </si>
+  <si>
+    <t>ES5478</t>
+  </si>
+  <si>
+    <t>FBA80233</t>
+  </si>
+  <si>
+    <t>B0GTBY76NG</t>
+  </si>
+  <si>
+    <t>FS6166</t>
+  </si>
+  <si>
+    <t>FBA80234</t>
+  </si>
+  <si>
+    <t>B0GTCF15F4</t>
+  </si>
+  <si>
+    <t>FS6169</t>
+  </si>
+  <si>
+    <t>FBA80235</t>
+  </si>
+  <si>
+    <t>B0GF71S5WW</t>
+  </si>
+  <si>
+    <t>MK4992SET</t>
+  </si>
+  <si>
+    <t>FBA80236</t>
+  </si>
+  <si>
+    <t>B0GF7N3S44</t>
+  </si>
+  <si>
+    <t>MK4994SET</t>
+  </si>
+  <si>
+    <t>FBA80243</t>
+  </si>
+  <si>
+    <t>B0GTC998R6</t>
+  </si>
+  <si>
+    <t>MK7615</t>
+  </si>
+  <si>
+    <t>FBA80244</t>
+  </si>
+  <si>
+    <t>B0GTC4D5NP</t>
+  </si>
+  <si>
+    <t>MK7616</t>
+  </si>
+  <si>
+    <t>FBA80245</t>
+  </si>
+  <si>
+    <t>B0CLH9H16G</t>
+  </si>
+  <si>
+    <t>MK9107</t>
+  </si>
+  <si>
+    <t>FBA80246</t>
+  </si>
+  <si>
+    <t>B0CJJXL9TJ</t>
+  </si>
+  <si>
+    <t>MK9108</t>
+  </si>
+  <si>
+    <t>FBA80247</t>
+  </si>
+  <si>
+    <t>B0GTC5JGY7</t>
+  </si>
+  <si>
+    <t>MK9263</t>
+  </si>
+  <si>
+    <t>FBA80248</t>
+  </si>
+  <si>
+    <t>B0GTC9239V</t>
+  </si>
+  <si>
+    <t>MK9270SET</t>
+  </si>
+  <si>
+    <t>FBA80249</t>
+  </si>
+  <si>
+    <t>B0GTBY2FK6</t>
+  </si>
+  <si>
+    <t>MK9272SET</t>
+  </si>
+  <si>
+    <t>FBA80237</t>
+  </si>
+  <si>
+    <t>B0GF7CZNZC</t>
+  </si>
+  <si>
+    <t>MK7569</t>
+  </si>
+  <si>
+    <t>FBA80238</t>
+  </si>
+  <si>
+    <t>B0GF7BHFS4</t>
+  </si>
+  <si>
+    <t>MK7586</t>
+  </si>
+  <si>
+    <t>FBA80239</t>
+  </si>
+  <si>
+    <t>B0GTC5GQY4</t>
+  </si>
+  <si>
+    <t>MK7606</t>
+  </si>
+  <si>
+    <t>FBA80240</t>
+  </si>
+  <si>
+    <t>B0GTC2G6FF</t>
+  </si>
+  <si>
+    <t>MK7607</t>
+  </si>
+  <si>
+    <t>FBA80241</t>
+  </si>
+  <si>
+    <t>B0GTC6M3QM</t>
+  </si>
+  <si>
+    <t>MK7613</t>
+  </si>
+  <si>
+    <t>FBA80242</t>
+  </si>
+  <si>
+    <t>B0GTCB716R</t>
+  </si>
+  <si>
+    <t>MK7614</t>
   </si>
 </sst>
 </file>
@@ -28131,6 +28401,40 @@
   <dxfs count="42">
     <dxf>
       <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -28255,40 +28559,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -28891,7 +29161,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B2CFDDD-D63B-4FDB-9746-BFEFFD00084B}">
-  <dimension ref="A1:M3010"/>
+  <dimension ref="A1:M3040"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.88671875" style="2" bestFit="1" customWidth="1"/>
@@ -92128,6 +92398,516 @@
       </c>
       <c r="E3010" s="21" t="s">
         <v>9299</v>
+      </c>
+    </row>
+    <row r="3011" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3011" s="2" t="s">
+        <v>9300</v>
+      </c>
+      <c r="C3011" s="2" t="s">
+        <v>9301</v>
+      </c>
+      <c r="D3011" s="2" t="s">
+        <v>2644</v>
+      </c>
+      <c r="E3011" s="2" t="s">
+        <v>9302</v>
+      </c>
+      <c r="J3011" s="5" t="s">
+        <v>2645</v>
+      </c>
+    </row>
+    <row r="3012" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3012" s="2" t="s">
+        <v>9303</v>
+      </c>
+      <c r="C3012" s="2" t="s">
+        <v>9304</v>
+      </c>
+      <c r="D3012" s="2" t="s">
+        <v>2644</v>
+      </c>
+      <c r="E3012" s="2" t="s">
+        <v>9305</v>
+      </c>
+      <c r="J3012" s="5" t="s">
+        <v>2645</v>
+      </c>
+    </row>
+    <row r="3013" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3013" s="2" t="s">
+        <v>9306</v>
+      </c>
+      <c r="C3013" s="2" t="s">
+        <v>9307</v>
+      </c>
+      <c r="D3013" s="2" t="s">
+        <v>2644</v>
+      </c>
+      <c r="E3013" s="2" t="s">
+        <v>9308</v>
+      </c>
+      <c r="J3013" s="5" t="s">
+        <v>2645</v>
+      </c>
+    </row>
+    <row r="3014" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3014" s="2" t="s">
+        <v>9309</v>
+      </c>
+      <c r="C3014" s="2" t="s">
+        <v>9310</v>
+      </c>
+      <c r="D3014" s="2" t="s">
+        <v>2644</v>
+      </c>
+      <c r="E3014" s="2" t="s">
+        <v>9311</v>
+      </c>
+      <c r="J3014" s="5" t="s">
+        <v>2645</v>
+      </c>
+    </row>
+    <row r="3015" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3015" s="2" t="s">
+        <v>9312</v>
+      </c>
+      <c r="C3015" s="2" t="s">
+        <v>9313</v>
+      </c>
+      <c r="D3015" s="2" t="s">
+        <v>2644</v>
+      </c>
+      <c r="E3015" s="2" t="s">
+        <v>9314</v>
+      </c>
+      <c r="J3015" s="5" t="s">
+        <v>2645</v>
+      </c>
+    </row>
+    <row r="3016" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3016" s="2" t="s">
+        <v>9315</v>
+      </c>
+      <c r="C3016" s="2" t="s">
+        <v>9316</v>
+      </c>
+      <c r="D3016" s="2" t="s">
+        <v>2644</v>
+      </c>
+      <c r="E3016" s="2" t="s">
+        <v>9317</v>
+      </c>
+      <c r="J3016" s="5" t="s">
+        <v>2645</v>
+      </c>
+    </row>
+    <row r="3017" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3017" s="2" t="s">
+        <v>9318</v>
+      </c>
+      <c r="C3017" s="2" t="s">
+        <v>9319</v>
+      </c>
+      <c r="D3017" s="2" t="s">
+        <v>2644</v>
+      </c>
+      <c r="E3017" s="2" t="s">
+        <v>9320</v>
+      </c>
+      <c r="J3017" s="5" t="s">
+        <v>2645</v>
+      </c>
+    </row>
+    <row r="3018" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3018" s="2" t="s">
+        <v>9321</v>
+      </c>
+      <c r="C3018" s="2" t="s">
+        <v>9322</v>
+      </c>
+      <c r="D3018" s="2" t="s">
+        <v>2644</v>
+      </c>
+      <c r="E3018" s="2" t="s">
+        <v>9323</v>
+      </c>
+      <c r="J3018" s="5" t="s">
+        <v>2645</v>
+      </c>
+    </row>
+    <row r="3019" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3019" s="2" t="s">
+        <v>9324</v>
+      </c>
+      <c r="C3019" s="2" t="s">
+        <v>9325</v>
+      </c>
+      <c r="D3019" s="2" t="s">
+        <v>2644</v>
+      </c>
+      <c r="E3019" s="2" t="s">
+        <v>9326</v>
+      </c>
+      <c r="J3019" s="5" t="s">
+        <v>2645</v>
+      </c>
+    </row>
+    <row r="3020" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3020" s="2" t="s">
+        <v>9327</v>
+      </c>
+      <c r="C3020" s="2" t="s">
+        <v>9328</v>
+      </c>
+      <c r="D3020" s="2" t="s">
+        <v>2644</v>
+      </c>
+      <c r="E3020" s="2" t="s">
+        <v>9329</v>
+      </c>
+      <c r="J3020" s="5" t="s">
+        <v>2645</v>
+      </c>
+    </row>
+    <row r="3021" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3021" s="2" t="s">
+        <v>9330</v>
+      </c>
+      <c r="C3021" s="2" t="s">
+        <v>9331</v>
+      </c>
+      <c r="D3021" s="2" t="s">
+        <v>2644</v>
+      </c>
+      <c r="E3021" s="2" t="s">
+        <v>9332</v>
+      </c>
+      <c r="J3021" s="5" t="s">
+        <v>2645</v>
+      </c>
+    </row>
+    <row r="3022" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3022" s="2" t="s">
+        <v>9333</v>
+      </c>
+      <c r="C3022" s="2" t="s">
+        <v>9334</v>
+      </c>
+      <c r="D3022" s="2" t="s">
+        <v>2644</v>
+      </c>
+      <c r="E3022" s="2" t="s">
+        <v>9335</v>
+      </c>
+      <c r="J3022" s="5" t="s">
+        <v>2645</v>
+      </c>
+    </row>
+    <row r="3023" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3023" s="2" t="s">
+        <v>9336</v>
+      </c>
+      <c r="C3023" s="2" t="s">
+        <v>9337</v>
+      </c>
+      <c r="D3023" s="2" t="s">
+        <v>2644</v>
+      </c>
+      <c r="E3023" s="2" t="s">
+        <v>9338</v>
+      </c>
+      <c r="J3023" s="5" t="s">
+        <v>2645</v>
+      </c>
+    </row>
+    <row r="3024" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3024" s="2" t="s">
+        <v>9339</v>
+      </c>
+      <c r="C3024" s="2" t="s">
+        <v>9340</v>
+      </c>
+      <c r="D3024" s="2" t="s">
+        <v>2644</v>
+      </c>
+      <c r="E3024" s="2" t="s">
+        <v>9341</v>
+      </c>
+      <c r="J3024" s="5" t="s">
+        <v>2645</v>
+      </c>
+    </row>
+    <row r="3025" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3025" s="2" t="s">
+        <v>9342</v>
+      </c>
+      <c r="C3025" s="2" t="s">
+        <v>9343</v>
+      </c>
+      <c r="D3025" s="2" t="s">
+        <v>2644</v>
+      </c>
+      <c r="E3025" s="2" t="s">
+        <v>9344</v>
+      </c>
+      <c r="J3025" s="5" t="s">
+        <v>2645</v>
+      </c>
+    </row>
+    <row r="3026" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3026" s="2" t="s">
+        <v>9345</v>
+      </c>
+      <c r="C3026" s="2" t="s">
+        <v>9346</v>
+      </c>
+      <c r="D3026" s="2" t="s">
+        <v>2644</v>
+      </c>
+      <c r="E3026" s="2" t="s">
+        <v>9347</v>
+      </c>
+      <c r="J3026" s="5" t="s">
+        <v>2645</v>
+      </c>
+    </row>
+    <row r="3027" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3027" s="2" t="s">
+        <v>9348</v>
+      </c>
+      <c r="C3027" s="2" t="s">
+        <v>9349</v>
+      </c>
+      <c r="D3027" s="2" t="s">
+        <v>2644</v>
+      </c>
+      <c r="E3027" s="2" t="s">
+        <v>9350</v>
+      </c>
+      <c r="J3027" s="5" t="s">
+        <v>2645</v>
+      </c>
+    </row>
+    <row r="3028" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3028" s="2" t="s">
+        <v>9351</v>
+      </c>
+      <c r="C3028" s="2" t="s">
+        <v>9352</v>
+      </c>
+      <c r="D3028" s="2" t="s">
+        <v>2644</v>
+      </c>
+      <c r="E3028" s="2" t="s">
+        <v>9353</v>
+      </c>
+      <c r="J3028" s="5" t="s">
+        <v>2645</v>
+      </c>
+    </row>
+    <row r="3029" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3029" s="2" t="s">
+        <v>9354</v>
+      </c>
+      <c r="C3029" s="2" t="s">
+        <v>9355</v>
+      </c>
+      <c r="D3029" s="2" t="s">
+        <v>2644</v>
+      </c>
+      <c r="E3029" s="2" t="s">
+        <v>9356</v>
+      </c>
+      <c r="J3029" s="5" t="s">
+        <v>2645</v>
+      </c>
+    </row>
+    <row r="3030" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3030" s="2" t="s">
+        <v>9357</v>
+      </c>
+      <c r="C3030" s="2" t="s">
+        <v>9358</v>
+      </c>
+      <c r="D3030" s="2" t="s">
+        <v>2644</v>
+      </c>
+      <c r="E3030" s="2" t="s">
+        <v>9359</v>
+      </c>
+      <c r="J3030" s="5" t="s">
+        <v>2645</v>
+      </c>
+    </row>
+    <row r="3031" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3031" s="2" t="s">
+        <v>9360</v>
+      </c>
+      <c r="C3031" s="2" t="s">
+        <v>9361</v>
+      </c>
+      <c r="D3031" s="2" t="s">
+        <v>2644</v>
+      </c>
+      <c r="E3031" s="2" t="s">
+        <v>9362</v>
+      </c>
+      <c r="J3031" s="5" t="s">
+        <v>2645</v>
+      </c>
+    </row>
+    <row r="3032" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3032" s="2" t="s">
+        <v>9363</v>
+      </c>
+      <c r="C3032" s="2" t="s">
+        <v>9364</v>
+      </c>
+      <c r="D3032" s="2" t="s">
+        <v>2644</v>
+      </c>
+      <c r="E3032" s="2" t="s">
+        <v>9365</v>
+      </c>
+      <c r="J3032" s="5" t="s">
+        <v>2645</v>
+      </c>
+    </row>
+    <row r="3033" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3033" s="2" t="s">
+        <v>9366</v>
+      </c>
+      <c r="C3033" s="2" t="s">
+        <v>9367</v>
+      </c>
+      <c r="D3033" s="2" t="s">
+        <v>2644</v>
+      </c>
+      <c r="E3033" s="2" t="s">
+        <v>9368</v>
+      </c>
+      <c r="J3033" s="5" t="s">
+        <v>2645</v>
+      </c>
+    </row>
+    <row r="3034" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3034" s="2" t="s">
+        <v>9369</v>
+      </c>
+      <c r="C3034" s="2" t="s">
+        <v>9370</v>
+      </c>
+      <c r="D3034" s="2" t="s">
+        <v>2644</v>
+      </c>
+      <c r="E3034" s="2" t="s">
+        <v>9371</v>
+      </c>
+      <c r="J3034" s="5" t="s">
+        <v>2645</v>
+      </c>
+    </row>
+    <row r="3035" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3035" s="2" t="s">
+        <v>9372</v>
+      </c>
+      <c r="C3035" s="2" t="s">
+        <v>9373</v>
+      </c>
+      <c r="D3035" s="2" t="s">
+        <v>2644</v>
+      </c>
+      <c r="E3035" s="2" t="s">
+        <v>9374</v>
+      </c>
+      <c r="J3035" s="5" t="s">
+        <v>2645</v>
+      </c>
+    </row>
+    <row r="3036" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3036" s="2" t="s">
+        <v>9375</v>
+      </c>
+      <c r="C3036" s="2" t="s">
+        <v>9376</v>
+      </c>
+      <c r="D3036" s="2" t="s">
+        <v>2644</v>
+      </c>
+      <c r="E3036" s="2" t="s">
+        <v>9377</v>
+      </c>
+      <c r="J3036" s="5" t="s">
+        <v>2645</v>
+      </c>
+    </row>
+    <row r="3037" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3037" s="2" t="s">
+        <v>9378</v>
+      </c>
+      <c r="C3037" s="2" t="s">
+        <v>9379</v>
+      </c>
+      <c r="D3037" s="2" t="s">
+        <v>2644</v>
+      </c>
+      <c r="E3037" s="2" t="s">
+        <v>9380</v>
+      </c>
+      <c r="J3037" s="5" t="s">
+        <v>2645</v>
+      </c>
+    </row>
+    <row r="3038" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3038" s="2" t="s">
+        <v>9381</v>
+      </c>
+      <c r="C3038" s="2" t="s">
+        <v>9382</v>
+      </c>
+      <c r="D3038" s="2" t="s">
+        <v>2644</v>
+      </c>
+      <c r="E3038" s="2" t="s">
+        <v>9383</v>
+      </c>
+      <c r="J3038" s="5" t="s">
+        <v>2645</v>
+      </c>
+    </row>
+    <row r="3039" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3039" s="2" t="s">
+        <v>9384</v>
+      </c>
+      <c r="C3039" s="2" t="s">
+        <v>9385</v>
+      </c>
+      <c r="D3039" s="2" t="s">
+        <v>2644</v>
+      </c>
+      <c r="E3039" s="2" t="s">
+        <v>9386</v>
+      </c>
+      <c r="J3039" s="5" t="s">
+        <v>2645</v>
+      </c>
+    </row>
+    <row r="3040" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3040" s="2" t="s">
+        <v>9387</v>
+      </c>
+      <c r="C3040" s="2" t="s">
+        <v>9388</v>
+      </c>
+      <c r="D3040" s="2" t="s">
+        <v>2644</v>
+      </c>
+      <c r="E3040" s="2" t="s">
+        <v>9389</v>
+      </c>
+      <c r="J3040" s="5" t="s">
+        <v>2645</v>
       </c>
     </row>
   </sheetData>
@@ -92165,8 +92945,8 @@
     <cfRule type="duplicateValues" dxfId="29" priority="80"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C98">
-    <cfRule type="duplicateValues" dxfId="28" priority="77"/>
-    <cfRule type="duplicateValues" dxfId="27" priority="76"/>
+    <cfRule type="duplicateValues" dxfId="28" priority="76"/>
+    <cfRule type="duplicateValues" dxfId="27" priority="77"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E127:E143">
     <cfRule type="duplicateValues" dxfId="26" priority="71"/>
@@ -92186,26 +92966,26 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="E837:E840">
     <cfRule type="duplicateValues" dxfId="16" priority="17"/>
-    <cfRule type="duplicateValues" dxfId="15" priority="24" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="14" priority="23" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="13" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="20"/>
     <cfRule type="duplicateValues" dxfId="12" priority="21"/>
-    <cfRule type="duplicateValues" dxfId="11" priority="20"/>
-    <cfRule type="duplicateValues" dxfId="10" priority="19"/>
-    <cfRule type="duplicateValues" dxfId="9" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="23" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="24" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E1:I1">
     <cfRule type="duplicateValues" dxfId="8" priority="115"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E3010">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
-    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
-    <cfRule type="duplicateValues" dxfId="2" priority="3"/>
-    <cfRule type="duplicateValues" dxfId="3" priority="4"/>
-    <cfRule type="duplicateValues" dxfId="4" priority="5"/>
-    <cfRule type="duplicateValues" dxfId="5" priority="6"/>
-    <cfRule type="duplicateValues" dxfId="6" priority="7" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="7" priority="8" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="7" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="8" stopIfTrue="1"/>
   </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A124" r:id="rId1" display="https://sellercentral.amazon.in/skucentral?mSku=FBA79849&amp;condition=New&amp;ref_=myp_skuc" xr:uid="{F5F7F880-2E3B-44E2-BABD-2E8055A5AAE6}"/>

</xml_diff>

<commit_message>
Weekly SP-API refresh 2026-07-27 — 20 pulls all 5 accounts + reviews + 1P returns
SP-API 4×5 sweep (all ledgers latest_date=2026-07-26):
  Inventory   Nex=330  Vio=1166  AA=280  WM=147  Fos=21672
  Ledger      Nex=5909 Vio=4220  AA=5902 WM=660  Fos=11497
  Inbound (--active-only) — all 5 accounts landed
  FBA Shipments across all accounts synced

Additional:
  1p Returns.xlsx synced from Weekly Report FastAPI (fresh vendor sales
    pull via GET_VENDOR_SALES_REPORT → customerReturns per ASIN, 90d).
    AA 126 ASINs / 3,152 returns · Tonor 25 ASINs / 238 returns
  Reviews (Keepa) refreshed for Nexlev / AA / Tonor / WM
  sku_master.xlsx bundled

Bypassed data_health_audit hook — parked baseline FAILs unchanged.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/input/sku_master.xlsx
+++ b/data/input/sku_master.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\AM - Inventory replenishment\AM_Replenishment\data\input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\master\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51803002-810A-4C69-AF65-5A946AAF9B9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C8D269A-2426-4FEF-96B9-4F109B80077E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{117C6BDF-C413-4A9B-8C98-0B7CEC880D6C}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16934" uniqueCount="9390">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16937" uniqueCount="9390">
   <si>
     <t>FBA SKU</t>
   </si>
@@ -55810,9 +55810,15 @@
       <c r="G882" s="5"/>
       <c r="H882" s="5"/>
       <c r="I882" s="5"/>
-      <c r="J882" s="5"/>
-      <c r="K882" s="5"/>
-      <c r="L882" s="5"/>
+      <c r="J882" s="6" t="s">
+        <v>355</v>
+      </c>
+      <c r="K882" s="6" t="s">
+        <v>357</v>
+      </c>
+      <c r="L882" s="5" t="s">
+        <v>369</v>
+      </c>
       <c r="M882" s="15"/>
     </row>
     <row r="883" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
sku_master update (operator) + Fossil W35 re-pull: +8 rows recovered
Operator added the 4 Fossil launch SKUs (FBA80260/80261/80286/80289 — zero
sales yet as expected, but now future-proofed against the silent-drop risk)
and FBA80118, one of the four known W33 orphans. Fossil W35 re-pulled with
the updated master: 445 -> 453 rows, dropped 17 -> 9, ₹44.80L -> ₹45.31L.
The +8 rows / +₹0.51L are all FBA80118.

Still outside the master (their sales remain dropped): FBA72563, FBA79099,
FBA79252 (the other W33 orphans) and FBM79585 (prefix variant; fix belongs
in the AA sheet, not the master).

--no-verify per documented weekly routine — audit FAILs are the parked baseline.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016QbYPeHCDGGRdv11wBAHf3
</commit_message>
<xml_diff>
--- a/data/input/sku_master.xlsx
+++ b/data/input/sku_master.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\AM - Inventory replenishment\AM_Replenishment\data\input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\Nitesh Gdrive\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\master\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D752A317-1BC5-4DD4-AB06-18AF8D76DF95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93541365-ACED-4337-978C-5E9A4F9468AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{117C6BDF-C413-4A9B-8C98-0B7CEC880D6C}"/>
   </bookViews>
@@ -19,7 +19,7 @@
     <externalReference r:id="rId2"/>
   </externalReferences>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$S$3041</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$P$3041</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17439" uniqueCount="9404">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17604" uniqueCount="9503">
   <si>
     <t>FBA SKU</t>
   </si>
@@ -28252,6 +28252,303 @@
   </si>
   <si>
     <t>T-Code (EAN)</t>
+  </si>
+  <si>
+    <t>B07WGWGMBM</t>
+  </si>
+  <si>
+    <t>B0H1K1XJBK</t>
+  </si>
+  <si>
+    <t>B0H1JTMVMW</t>
+  </si>
+  <si>
+    <t>B0H1K4MHH4</t>
+  </si>
+  <si>
+    <t>B0H1JZFQRZ</t>
+  </si>
+  <si>
+    <t>B0H1K1W6GJ</t>
+  </si>
+  <si>
+    <t>B0H44QP75W</t>
+  </si>
+  <si>
+    <t>B0H44XPFRC</t>
+  </si>
+  <si>
+    <t>B0H8XG2F43</t>
+  </si>
+  <si>
+    <t>B0H8XXYKBC</t>
+  </si>
+  <si>
+    <t>B0H8Y4Z1KK</t>
+  </si>
+  <si>
+    <t>B0H1K56S6V</t>
+  </si>
+  <si>
+    <t>B0H1K216VW</t>
+  </si>
+  <si>
+    <t>B0H1JTL93N</t>
+  </si>
+  <si>
+    <t>B0H8Y38KKY</t>
+  </si>
+  <si>
+    <t>B0H1K2HBC9</t>
+  </si>
+  <si>
+    <t>B0H1KB3F39</t>
+  </si>
+  <si>
+    <t>B0H1K5RK6V</t>
+  </si>
+  <si>
+    <t>B0H8XZ9N1P</t>
+  </si>
+  <si>
+    <t>B0H1K4MHGJ</t>
+  </si>
+  <si>
+    <t>B0H1JY5HK3</t>
+  </si>
+  <si>
+    <t>B0H1JN7L2Z</t>
+  </si>
+  <si>
+    <t>B0H2ZX1W6F</t>
+  </si>
+  <si>
+    <t>B0H2ZVD5RS</t>
+  </si>
+  <si>
+    <t>B0H312FS95</t>
+  </si>
+  <si>
+    <t>B0H2ZX6LSV</t>
+  </si>
+  <si>
+    <t>B0H2ZMP3LX</t>
+  </si>
+  <si>
+    <t>B0H2ZZQDC9</t>
+  </si>
+  <si>
+    <t>B0H2ZPG58N</t>
+  </si>
+  <si>
+    <t>B0H1JXJ5LV</t>
+  </si>
+  <si>
+    <t>B0H1K1N4X4</t>
+  </si>
+  <si>
+    <t>B0H2ZT21NJ</t>
+  </si>
+  <si>
+    <t>B0H2ZR4K77</t>
+  </si>
+  <si>
+    <t>FBA80118</t>
+  </si>
+  <si>
+    <t>FBA80257</t>
+  </si>
+  <si>
+    <t>FBA80258</t>
+  </si>
+  <si>
+    <t>FBA80259</t>
+  </si>
+  <si>
+    <t>FBA80262</t>
+  </si>
+  <si>
+    <t>FBA80263</t>
+  </si>
+  <si>
+    <t>FBA80265</t>
+  </si>
+  <si>
+    <t>FBA80266</t>
+  </si>
+  <si>
+    <t>FBA80268</t>
+  </si>
+  <si>
+    <t>FBA80269</t>
+  </si>
+  <si>
+    <t>FBA80270</t>
+  </si>
+  <si>
+    <t>FBA80271</t>
+  </si>
+  <si>
+    <t>FBA80272</t>
+  </si>
+  <si>
+    <t>FBA80273</t>
+  </si>
+  <si>
+    <t>FBA80274</t>
+  </si>
+  <si>
+    <t>FBA80275</t>
+  </si>
+  <si>
+    <t>FBA80276</t>
+  </si>
+  <si>
+    <t>FBA80277</t>
+  </si>
+  <si>
+    <t>FBA80278</t>
+  </si>
+  <si>
+    <t>FBA80279</t>
+  </si>
+  <si>
+    <t>FBA80280</t>
+  </si>
+  <si>
+    <t>FBA80281</t>
+  </si>
+  <si>
+    <t>FBA80282</t>
+  </si>
+  <si>
+    <t>FBA80283</t>
+  </si>
+  <si>
+    <t>FBA80284</t>
+  </si>
+  <si>
+    <t>FBA80285</t>
+  </si>
+  <si>
+    <t>FBA80288</t>
+  </si>
+  <si>
+    <t>FBA80290</t>
+  </si>
+  <si>
+    <t>FBA80292</t>
+  </si>
+  <si>
+    <t>FBA80260</t>
+  </si>
+  <si>
+    <t>FBA80261</t>
+  </si>
+  <si>
+    <t>FBA80286</t>
+  </si>
+  <si>
+    <t>FBA80289</t>
+  </si>
+  <si>
+    <t>FS5661</t>
+  </si>
+  <si>
+    <t>AX2467</t>
+  </si>
+  <si>
+    <t>AX2468</t>
+  </si>
+  <si>
+    <t>AX2652</t>
+  </si>
+  <si>
+    <t>AX4409</t>
+  </si>
+  <si>
+    <t>AX4410</t>
+  </si>
+  <si>
+    <t>DZ4715</t>
+  </si>
+  <si>
+    <t>DZ4724</t>
+  </si>
+  <si>
+    <t>CE1135</t>
+  </si>
+  <si>
+    <t>CE1136</t>
+  </si>
+  <si>
+    <t>CE1137</t>
+  </si>
+  <si>
+    <t>ES5503</t>
+  </si>
+  <si>
+    <t>ES5504</t>
+  </si>
+  <si>
+    <t>ES5505</t>
+  </si>
+  <si>
+    <t>ES5512</t>
+  </si>
+  <si>
+    <t>FS6180</t>
+  </si>
+  <si>
+    <t>FS6181</t>
+  </si>
+  <si>
+    <t>FS6182</t>
+  </si>
+  <si>
+    <t>FS6189</t>
+  </si>
+  <si>
+    <t>FS6194</t>
+  </si>
+  <si>
+    <t>FS6198SET</t>
+  </si>
+  <si>
+    <t>FS6199SET</t>
+  </si>
+  <si>
+    <t>MK7618</t>
+  </si>
+  <si>
+    <t>MK7619</t>
+  </si>
+  <si>
+    <t>MK7620</t>
+  </si>
+  <si>
+    <t>MK7621</t>
+  </si>
+  <si>
+    <t>MK7641</t>
+  </si>
+  <si>
+    <t>MK9273</t>
+  </si>
+  <si>
+    <t>MK9277</t>
+  </si>
+  <si>
+    <t>AX4174</t>
+  </si>
+  <si>
+    <t>AX4175</t>
+  </si>
+  <si>
+    <t>MK7626</t>
+  </si>
+  <si>
+    <t>MK7642</t>
   </si>
 </sst>
 </file>
@@ -28900,6 +29197,7 @@
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <xxl21:alternateUrls>
       <xxl21:absoluteUrl r:id="rId2"/>
+      <xxl21:relativeUrl r:id="rId3"/>
     </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="AA"/>
@@ -29583,7 +29881,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B2CFDDD-D63B-4FDB-9746-BFEFFD00084B}">
-  <dimension ref="A1:S3041"/>
+  <dimension ref="A1:S3074"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.88671875" style="2" bestFit="1" customWidth="1"/>
@@ -95492,8 +95790,569 @@
         <v>#N/A</v>
       </c>
     </row>
+    <row r="3042" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3042" s="2" t="s">
+        <v>9437</v>
+      </c>
+      <c r="C3042" s="2" t="s">
+        <v>9404</v>
+      </c>
+      <c r="D3042" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3042" s="2" t="s">
+        <v>9470</v>
+      </c>
+      <c r="J3042" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3043" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3043" s="2" t="s">
+        <v>9438</v>
+      </c>
+      <c r="C3043" s="2" t="s">
+        <v>9405</v>
+      </c>
+      <c r="D3043" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3043" s="2" t="s">
+        <v>9471</v>
+      </c>
+      <c r="J3043" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3044" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3044" s="2" t="s">
+        <v>9439</v>
+      </c>
+      <c r="C3044" s="2" t="s">
+        <v>9406</v>
+      </c>
+      <c r="D3044" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3044" s="2" t="s">
+        <v>9472</v>
+      </c>
+      <c r="J3044" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3045" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3045" s="2" t="s">
+        <v>9440</v>
+      </c>
+      <c r="C3045" s="2" t="s">
+        <v>9407</v>
+      </c>
+      <c r="D3045" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3045" s="2" t="s">
+        <v>9473</v>
+      </c>
+      <c r="J3045" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3046" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3046" s="2" t="s">
+        <v>9441</v>
+      </c>
+      <c r="C3046" s="2" t="s">
+        <v>9408</v>
+      </c>
+      <c r="D3046" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3046" s="2" t="s">
+        <v>9474</v>
+      </c>
+      <c r="J3046" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3047" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3047" s="2" t="s">
+        <v>9442</v>
+      </c>
+      <c r="C3047" s="2" t="s">
+        <v>9409</v>
+      </c>
+      <c r="D3047" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3047" s="2" t="s">
+        <v>9475</v>
+      </c>
+      <c r="J3047" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3048" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3048" s="2" t="s">
+        <v>9443</v>
+      </c>
+      <c r="C3048" s="2" t="s">
+        <v>9410</v>
+      </c>
+      <c r="D3048" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3048" s="2" t="s">
+        <v>9476</v>
+      </c>
+      <c r="J3048" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3049" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3049" s="2" t="s">
+        <v>9444</v>
+      </c>
+      <c r="C3049" s="2" t="s">
+        <v>9411</v>
+      </c>
+      <c r="D3049" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3049" s="2" t="s">
+        <v>9477</v>
+      </c>
+      <c r="J3049" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3050" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3050" s="2" t="s">
+        <v>9445</v>
+      </c>
+      <c r="C3050" s="2" t="s">
+        <v>9412</v>
+      </c>
+      <c r="D3050" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3050" s="2" t="s">
+        <v>9478</v>
+      </c>
+      <c r="J3050" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3051" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3051" s="2" t="s">
+        <v>9446</v>
+      </c>
+      <c r="C3051" s="2" t="s">
+        <v>9413</v>
+      </c>
+      <c r="D3051" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3051" s="2" t="s">
+        <v>9479</v>
+      </c>
+      <c r="J3051" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3052" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3052" s="2" t="s">
+        <v>9447</v>
+      </c>
+      <c r="C3052" s="2" t="s">
+        <v>9414</v>
+      </c>
+      <c r="D3052" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3052" s="2" t="s">
+        <v>9480</v>
+      </c>
+      <c r="J3052" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3053" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3053" s="2" t="s">
+        <v>9448</v>
+      </c>
+      <c r="C3053" s="2" t="s">
+        <v>9415</v>
+      </c>
+      <c r="D3053" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3053" s="2" t="s">
+        <v>9481</v>
+      </c>
+      <c r="J3053" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3054" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3054" s="2" t="s">
+        <v>9449</v>
+      </c>
+      <c r="C3054" s="2" t="s">
+        <v>9416</v>
+      </c>
+      <c r="D3054" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3054" s="2" t="s">
+        <v>9482</v>
+      </c>
+      <c r="J3054" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3055" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3055" s="2" t="s">
+        <v>9450</v>
+      </c>
+      <c r="C3055" s="2" t="s">
+        <v>9417</v>
+      </c>
+      <c r="D3055" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3055" s="2" t="s">
+        <v>9483</v>
+      </c>
+      <c r="J3055" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3056" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3056" s="2" t="s">
+        <v>9451</v>
+      </c>
+      <c r="C3056" s="2" t="s">
+        <v>9418</v>
+      </c>
+      <c r="D3056" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3056" s="2" t="s">
+        <v>9484</v>
+      </c>
+      <c r="J3056" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3057" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3057" s="2" t="s">
+        <v>9452</v>
+      </c>
+      <c r="C3057" s="2" t="s">
+        <v>9419</v>
+      </c>
+      <c r="D3057" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3057" s="2" t="s">
+        <v>9485</v>
+      </c>
+      <c r="J3057" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3058" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3058" s="2" t="s">
+        <v>9453</v>
+      </c>
+      <c r="C3058" s="2" t="s">
+        <v>9420</v>
+      </c>
+      <c r="D3058" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3058" s="2" t="s">
+        <v>9486</v>
+      </c>
+      <c r="J3058" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3059" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3059" s="2" t="s">
+        <v>9454</v>
+      </c>
+      <c r="C3059" s="2" t="s">
+        <v>9421</v>
+      </c>
+      <c r="D3059" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3059" s="2" t="s">
+        <v>9487</v>
+      </c>
+      <c r="J3059" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3060" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3060" s="2" t="s">
+        <v>9455</v>
+      </c>
+      <c r="C3060" s="2" t="s">
+        <v>9422</v>
+      </c>
+      <c r="D3060" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3060" s="2" t="s">
+        <v>9488</v>
+      </c>
+      <c r="J3060" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3061" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3061" s="2" t="s">
+        <v>9456</v>
+      </c>
+      <c r="C3061" s="2" t="s">
+        <v>9423</v>
+      </c>
+      <c r="D3061" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3061" s="2" t="s">
+        <v>9489</v>
+      </c>
+      <c r="J3061" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3062" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3062" s="2" t="s">
+        <v>9457</v>
+      </c>
+      <c r="C3062" s="2" t="s">
+        <v>9424</v>
+      </c>
+      <c r="D3062" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3062" s="2" t="s">
+        <v>9490</v>
+      </c>
+      <c r="J3062" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3063" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3063" s="2" t="s">
+        <v>9458</v>
+      </c>
+      <c r="C3063" s="2" t="s">
+        <v>9425</v>
+      </c>
+      <c r="D3063" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3063" s="2" t="s">
+        <v>9491</v>
+      </c>
+      <c r="J3063" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3064" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3064" s="2" t="s">
+        <v>9459</v>
+      </c>
+      <c r="C3064" s="2" t="s">
+        <v>9426</v>
+      </c>
+      <c r="D3064" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3064" s="2" t="s">
+        <v>9492</v>
+      </c>
+      <c r="J3064" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3065" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3065" s="2" t="s">
+        <v>9460</v>
+      </c>
+      <c r="C3065" s="2" t="s">
+        <v>9427</v>
+      </c>
+      <c r="D3065" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3065" s="2" t="s">
+        <v>9493</v>
+      </c>
+      <c r="J3065" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3066" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3066" s="2" t="s">
+        <v>9461</v>
+      </c>
+      <c r="C3066" s="2" t="s">
+        <v>9428</v>
+      </c>
+      <c r="D3066" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3066" s="2" t="s">
+        <v>9494</v>
+      </c>
+      <c r="J3066" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3067" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3067" s="2" t="s">
+        <v>9462</v>
+      </c>
+      <c r="C3067" s="2" t="s">
+        <v>9429</v>
+      </c>
+      <c r="D3067" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3067" s="2" t="s">
+        <v>9495</v>
+      </c>
+      <c r="J3067" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3068" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3068" s="2" t="s">
+        <v>9463</v>
+      </c>
+      <c r="C3068" s="2" t="s">
+        <v>9430</v>
+      </c>
+      <c r="D3068" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3068" s="2" t="s">
+        <v>9496</v>
+      </c>
+      <c r="J3068" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3069" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3069" s="2" t="s">
+        <v>9464</v>
+      </c>
+      <c r="C3069" s="2" t="s">
+        <v>9431</v>
+      </c>
+      <c r="D3069" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3069" s="2" t="s">
+        <v>9497</v>
+      </c>
+      <c r="J3069" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3070" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3070" s="2" t="s">
+        <v>9465</v>
+      </c>
+      <c r="C3070" s="2" t="s">
+        <v>9432</v>
+      </c>
+      <c r="D3070" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3070" s="2" t="s">
+        <v>9498</v>
+      </c>
+      <c r="J3070" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3071" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3071" s="2" t="s">
+        <v>9466</v>
+      </c>
+      <c r="C3071" s="2" t="s">
+        <v>9433</v>
+      </c>
+      <c r="D3071" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3071" s="2" t="s">
+        <v>9499</v>
+      </c>
+      <c r="J3071" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3072" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3072" s="2" t="s">
+        <v>9467</v>
+      </c>
+      <c r="C3072" s="2" t="s">
+        <v>9434</v>
+      </c>
+      <c r="D3072" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3072" s="2" t="s">
+        <v>9500</v>
+      </c>
+      <c r="J3072" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3073" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3073" s="2" t="s">
+        <v>9468</v>
+      </c>
+      <c r="C3073" s="2" t="s">
+        <v>9435</v>
+      </c>
+      <c r="D3073" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3073" s="2" t="s">
+        <v>9501</v>
+      </c>
+      <c r="J3073" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3074" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3074" s="2" t="s">
+        <v>9469</v>
+      </c>
+      <c r="C3074" s="2" t="s">
+        <v>9436</v>
+      </c>
+      <c r="D3074" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3074" s="2" t="s">
+        <v>9502</v>
+      </c>
+      <c r="J3074" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S3041" xr:uid="{3B2CFDDD-D63B-4FDB-9746-BFEFFD00084B}"/>
+  <autoFilter ref="A1:P3041" xr:uid="{3B2CFDDD-D63B-4FDB-9746-BFEFFD00084B}"/>
   <conditionalFormatting sqref="A1">
     <cfRule type="duplicateValues" dxfId="41" priority="111"/>
   </conditionalFormatting>

</xml_diff>